<commit_message>
data: update content.xlsx and regenerate events
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/content.xlsx
+++ b/docs/content.xlsx
@@ -13,14 +13,41 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={16ff7efc-bb06-4ebf-bbdf-5f8120576e3d}</author>
-    <author>tc={3e40ec33-6cf3-4a33-afbb-39168adff873}</author>
-    <author>tc={a36b1086-4032-47ad-bcee-8aaf3679ff8f}</author>
-    <author>tc={c996986f-a217-4480-9d9a-df812f454965}</author>
-    <author>tc={de50ee63-2068-45ae-a900-546a2f628472}</author>
+    <author>tc={05187ace-a827-4e19-a48d-f90aa28b5106}</author>
+    <author>tc={4cb305d8-e3a5-4c11-9396-5e2500af0dcf}</author>
+    <author>tc={4ee14459-0c2c-4c6e-95a6-49dd0ac33994}</author>
+    <author>tc={da276ba1-998a-4cb2-a067-37f7d629c1c0}</author>
+    <author>tc={ed0e8a67-ea1c-430f-a164-aff19c26a351}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{16ff7efc-bb06-4ebf-bbdf-5f8120576e3d}" ref="B31">
+    <comment authorId="0" xr:uid="{05187ace-a827-4e19-a48d-f90aa28b5106}" ref="A21">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	phần này thấy có nhiều hội nghị, ngày, mình tìm thông tin về ngày tháng bắt đầu  kết thúc hội nghị nhé, thay vì chỉ dừng ở năm
+</t>
+      </text>
+    </comment>
+    <comment authorId="1" xr:uid="{4cb305d8-e3a5-4c11-9396-5e2500af0dcf}" ref="B3">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	chỗ nào mà lấy được ngày tháng bắt đầu kết thúc thì add vào nhé, đừng chỉ dừng ở mỗi năm
+</t>
+      </text>
+    </comment>
+    <comment authorId="2" xr:uid="{4ee14459-0c2c-4c6e-95a6-49dd0ac33994}" ref="B22">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	phần này thấy có nhiều hội nghị, ngày, mình tìm thông tin về ngày tháng bắt đầu kết thúc hội nghị nhé, thay vì chỉ dừng ở năm
+</t>
+      </text>
+    </comment>
+    <comment authorId="3" xr:uid="{da276ba1-998a-4cb2-a067-37f7d629c1c0}" ref="B31">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -31,7 +58,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="1" xr:uid="{3e40ec33-6cf3-4a33-afbb-39168adff873}" ref="A1">
+    <comment authorId="4" xr:uid="{ed0e8a67-ea1c-430f-a164-aff19c26a351}" ref="A1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -42,39 +69,12 @@
 </t>
       </text>
     </comment>
-    <comment authorId="2" xr:uid="{a36b1086-4032-47ad-bcee-8aaf3679ff8f}" ref="B3">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	chỗ nào mà lấy được ngày tháng bắt đầu kết thúc thì add vào nhé, đừng chỉ dừng ở mỗi năm
-</t>
-      </text>
-    </comment>
-    <comment authorId="3" xr:uid="{c996986f-a217-4480-9d9a-df812f454965}" ref="A21">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	phần này thấy có nhiều hội nghị, ngày, mình tìm thông tin về ngày tháng bắt đầu  kết thúc hội nghị nhé, thay vì chỉ dừng ở năm
-</t>
-      </text>
-    </comment>
-    <comment authorId="4" xr:uid="{de50ee63-2068-45ae-a900-546a2f628472}" ref="B22">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	phần này thấy có nhiều hội nghị, ngày, mình tìm thông tin về ngày tháng bắt đầu kết thúc hội nghị nhé, thay vì chỉ dừng ở năm
-</t>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="217">
   <si>
     <t>STT</t>
   </si>
@@ -122,10 +122,10 @@
     <t>Đây là các cuộc đấu tranh lớn của thợ dệt lụa Lyon. Phong trào nêu yêu sách kinh tế về tiền công, điều kiện sống, đồng thời thể hiện bước phát triển về ý thức chính trị của giai cấp công nhân. Đây thường được xem là một trong những cuộc đấu tranh công nhân tiêu biểu đầu thế kỷ XIX.</t>
   </si>
   <si>
-    <t>https://en.wikipedia.org/wiki/Canut_revolts?utm_source=chatgpt.com</t>
+    <t>https://www.gadagne-lyon.fr/sites/gadagne/files/medias/documents/2020-12/MHL-Gadagne_ThemedSheet_19th-TheCanutRevolts.pdf?utm_source=chatgpt.com</t>
   </si>
   <si>
-    <t>https://commons.wikimedia.org/wiki/File:Revolte_des_Canuts_-_Lyon_1831_-_1.jpg</t>
+    <t>https://upload.wikimedia.org/wikipedia/commons/4/45/Revolte_des_Canuts_-_Lyon_1831_-_1.jpg</t>
   </si>
   <si>
     <t>1836 – 10/04/1848</t>
@@ -146,7 +146,7 @@
     <t>https://www.nationalarchives.gov.uk/education/resources/what-was-chartism/?utm_source=chatgpt.com</t>
   </si>
   <si>
-    <t>https://commons.wikimedia.org/wiki/File:Chartist_meeting,_Kennington_Common.jpg</t>
+    <t>https://upload.wikimedia.org/wikipedia/commons/2/24/Chartist_meeting%2C_Kennington_Common.jpg</t>
   </si>
   <si>
     <t>04/06/1844 – 06/06/1844</t>
@@ -167,7 +167,7 @@
     <t>https://www.deutschlandmuseum.de/en/history/calendar/1844-06-04-the-weavers-revolt/?utm_source=chatgpt.com</t>
   </si>
   <si>
-    <t>https://commons.wikimedia.org/wiki/File:Carl_Wilhelm_H%C3%BCbner_-_The_Silesian_Weavers_-_Google_Art_Project.jpg</t>
+    <t>https://upload.wikimedia.org/wikipedia/commons/9/9f/Carl_Wilhelm_H%C3%BCbner_-_The_Silesian_Weavers_-_Google_Art_Project.jpg</t>
   </si>
   <si>
     <t>Năm 1843 - 1844</t>
@@ -186,10 +186,10 @@
     <t>Giai đoạn này Mác và Ăngghen chuyển từ lập trường dân chủ cách mạng sang lập trường cộng sản. Mác nghiên cứu sâu về triết học, chính trị và kinh tế; Ăngghen nghiên cứu thực tiễn đời sống giai cấp công nhân ở Anh. Năm 1844, hai ông bắt đầu hợp tác chặt chẽ tại Paris, tạo tiền đề cho sự hình thành CNXHKH.</t>
   </si>
   <si>
-    <t>https://en.wikipedia.org/wiki/Friedrich_Engels?utm_source=chatgpt.com</t>
+    <t>https://thinhvuongvietnam.com/Content/ky-niem-202-nam-ngay-sinh-cmac-551818---552020-cmac-va-hanh-trinh-den-voi-chu-nghia-cong-san-31623?utm_source=chatgpt.com</t>
   </si>
   <si>
-    <t>https://commons.wikimedia.org/wiki/File:Marx_and_Engels.jpg</t>
+    <t>https://upload.wikimedia.org/wikipedia/commons/7/79/Marx_and_Engels.jpg</t>
   </si>
   <si>
     <t>2/1848</t>
@@ -207,7 +207,10 @@
     <t>Tác phẩm do C. Mác và Ph. Ăngghen soạn thảo, được công bố lần đầu bằng tiếng Đức vào tháng 2/1848 tại London. Tác phẩm đánh dấu sự ra đời về mặt lý luận của chủ nghĩa xã hội khoa học.</t>
   </si>
   <si>
-    <t>https://commons.wikimedia.org/wiki/File:Communist-manifesto.png</t>
+    <t>https://tulieuvankien.dangcongsan.vn/ho-so-su-kien-nhan-chung/su-kien-va-nhan-chung/tuyen-ngon-dang-cong-san-thang-2-1848-3385?utm_source=chatgpt.com</t>
+  </si>
+  <si>
+    <t>https://upload.wikimedia.org/wikipedia/commons/thumb/8/86/Communist-manifesto.png/500px-Communist-manifesto.png?_=20251104221727</t>
   </si>
   <si>
     <t>Năm 1848 - 1852</t>
@@ -225,10 +228,10 @@
     <t>Cách mạng 1848 thường được gọi là “Mùa xuân của các dân tộc”, bắt đầu lan rộng ở châu Âu từ năm 1848, tiêu biểu tại Pháp, Đức, Áo, Ý. Trong học phần, mốc 1848–1852 có thể hiểu là giai đoạn diễn ra, thất bại và được Mác – Ăngghen tổng kết kinh nghiệm cách mạng.</t>
   </si>
   <si>
-    <t>https://en.wikipedia.org/wiki/Revolutions_of_1848?utm_source=chatgpt.com</t>
+    <t>https://www.history.com/a-year-in-history/1848?utm_source=chatgpt.com</t>
   </si>
   <si>
-    <t>https://commons.wikimedia.org/wiki/File:Barricades_rue_Saint-Maur._Avant_l%27attaque,_25_juin_1848._Apr%C3%A8s_l%E2%80%99attaque,_26_juin_1848.jpg</t>
+    <t>https://upload.wikimedia.org/wikipedia/commons/thumb/2/26/Barricades_rue_Saint-Maur._Avant_l%27attaque%2C_25_juin_1848._Apr%C3%A8s_l%E2%80%99attaque%2C_26_juin_1848.jpg/960px-Barricades_rue_Saint-Maur._Avant_l%27attaque%2C_25_juin_1848._Apr%C3%A8s_l%E2%80%99attaque%2C_26_juin_1848.jpg?_=20230922071523</t>
   </si>
   <si>
     <t>28/09/1864</t>
@@ -246,7 +249,7 @@
     <t>Ngày 28/9/1864, Hội Liên hiệp Công nhân Quốc tế, thường gọi là Quốc tế I, được thành lập tại St Martin’s Hall, London. Tổ chức này góp phần liên kết phong trào công nhân quốc tế.</t>
   </si>
   <si>
-    <t>https://en.wikipedia.org/wiki/First_International?utm_source=chatgpt.com</t>
+    <t>https://tulieuvankien.dangcongsan.vn/ho-so-su-kien-nhan-chung/phong-trao-cong-san-cong-nhan-quoc-te/quoc-te-cong-san/quoc-te-i-1864-1876-103?utm_source=chatgpt.com</t>
   </si>
   <si>
     <t>14/09/1867</t>
@@ -264,7 +267,10 @@
     <t>Tập I của bộ Tư bản do C. Mác viết, xuất bản lần đầu bằng tiếng Đức tại Hamburg bởi nhà xuất bản Otto Meissner năm 1867. Đây là tác phẩm phân tích sâu sắc phương thức sản xuất tư bản chủ nghĩa.</t>
   </si>
   <si>
-    <t>https://commons.wikimedia.org/wiki/File:Marx_-_Das_Kapital_-_1867_-_DHM.JPG</t>
+    <t>https://germanhistorydocs.org/en/forging-an-empire-bismarckian-germany-1866-1890/karl-marx-capital-das-kapital-cover-of-the-1st-edition-1867?utm_source=chatgpt.com</t>
+  </si>
+  <si>
+    <t>https://upload.wikimedia.org/wikipedia/commons/d/da/Marx_-_Das_Kapital_-_1867_-_DHM.JPG</t>
   </si>
   <si>
     <t>18/03/1871 – 28/05/1871</t>
@@ -282,10 +288,10 @@
     <t>Công xã Paris tồn tại từ 18/3 đến 28/5/1871. Đây là chính quyền cách mạng của nhân dân lao động Paris, thường được xem là hình thức nhà nước mới đầu tiên của giai cấp công nhân.</t>
   </si>
   <si>
-    <t>https://en.wikipedia.org/wiki/Paris_Commune?utm_source=chatgpt.com</t>
+    <t>https://www.quanlynhanuoc.vn/2024/06/18/cong-xa-pari-mo-hinh-nha-nuoc-vo-san-dau-tien-va-y-nghia-doi-voi-xay-dung-nha-nuoc-phap-quyen-xa-hoi-chu-nghia-o-viet-nam-hien-nay/</t>
   </si>
   <si>
-    <t>https://commons.wikimedia.org/wiki/Category:Paris_Commune</t>
+    <t>https://upload.wikimedia.org/wikipedia/commons/thumb/b/bc/Barricade_de_la_rue_de_Flandre_%28_Salle_de_la_Marseillaise%29%2C_18_mars_1871._PH4142-167%281%29.jpg/250px-Barricade_de_la_rue_de_Flandre_%28_Salle_de_la_Marseillaise%29%2C_18_mars_1871._PH4142-167%281%29.jpg</t>
   </si>
   <si>
     <t>Năm 1875</t>
@@ -303,7 +309,10 @@
     <t>Tác phẩm được Mác viết vào tháng 4 hoặc đầu tháng 5/1875 để phê phán dự thảo cương lĩnh của đảng công nhân Đức trước Đại hội Gotha. Nội dung có ý nghĩa quan trọng trong việc làm rõ quan điểm của chủ nghĩa Mác về nhà nước, phân phối và thời kỳ quá độ.</t>
   </si>
   <si>
-    <t>https://commons.wikimedia.org/wiki/File:Karl_Marx._On_the_Critique_of_the_Social_Democratic_Party_Platform.png</t>
+    <t>https://tulieuvankien.dangcongsan.vn/c-mac-angghen-lenin-ho-chi-minh/c-mac/nghien-cuu-hoc-tap-tu-tuong/gia-tri-tu-tuong-cua-chu-nghia-mac-mai-truong-ton-3700</t>
+  </si>
+  <si>
+    <t>https://upload.wikimedia.org/wikipedia/commons/thumb/3/3e/Karl_Marx._On_the_Critique_of_the_Social_Democratic_Party_Platform.png/500px-Karl_Marx._On_the_Critique_of_the_Social_Democratic_Party_Platform.png?_=20251014223013</t>
   </si>
   <si>
     <t>Năm 1878</t>
@@ -321,7 +330,10 @@
     <t>“Chống Đuyrinh” do Ph. Ăngghen viết trong giai đoạn 1876–1878, đăng nhiều kỳ trên báo Vorwärts và xuất bản thành sách tại Leipzig năm 1878. Tác phẩm trình bày có hệ thống nhiều nội dung cơ bản của chủ nghĩa Mác.</t>
   </si>
   <si>
-    <t>https://commons.wikimedia.org/wiki/File:Anti_Duhring_cover.jpg</t>
+    <t>https://luatminhkhue.vn/gioi-thieu-khai-quat-tac-pham-chong-duyrinh-cua-ph-angghen.aspx</t>
+  </si>
+  <si>
+    <t>https://upload.wikimedia.org/wikipedia/commons/thumb/3/3a/Anti_Duhring_cover.jpg/500px-Anti_Duhring_cover.jpg?_=20260205183536</t>
   </si>
   <si>
     <t>Thời kỳ V.I. Lênin vận dụng và phát triển (Đầu thế kỷ XX) - Hưng</t>
@@ -499,6 +511,9 @@
     <t>https://vi.wikipedia.org/wiki/Chi%E1%BA%BFn_tranh_th%E1%BA%BF_gi%E1%BB%9Bi_th%E1%BB%A9_hai</t>
   </si>
   <si>
+    <t>https://vi.wikipedia.org/wiki/%C4%90%E1%BA%A1i_h%E1%BB%99i_%C4%90%E1%BA%A3ng_C%E1%BB%99ng_s%E1%BA%A3n_Trung_Qu%E1%BB%91c_l%E1%BA%A7n_th%E1%BB%A9_XVI</t>
+  </si>
+  <si>
     <t>Tháng 11/1957</t>
   </si>
   <si>
@@ -516,7 +531,7 @@
 </t>
   </si>
   <si>
-    <t>https://tulieuvankien.dangcongsan.vn/publish/thumbnail/3000006/600x315xdefault/upload/3000006/20251024/dad2668a506ae01795ec89e7b03f769016-1509940896360.jpg</t>
+    <t>https://hochiminh-image.nhandan.vn/t460/Uploaded/tgshzb/2022_05_06/17-12-1960_phong_trao_cong_san_va_cong_nhan___.jpg</t>
   </si>
   <si>
     <t>Tháng 1/1960</t>
@@ -529,7 +544,10 @@
 - Hội nghị thông qua bản Tuyên ngôn mới, bổ sung và phát triển nội dung Tuyên ngôn năm 1957, được coi là cương lĩnh cách mạng chung cho các Đảng Mác – Lênin trên thế giới</t>
   </si>
   <si>
-    <t>https://special.nhandan.vn/phong-trao-cong-san-va-cong-nhan-quoc-te-doan-ket-dau-tranh-thang-loi/index.html</t>
+    <t>https://tulieuvankien.dangcongsan.vn/ho-so-su-kien-nhan-chung/su-kien-va-nhan-chung/hoi-nghi-dai-bieu-cac-dang-cong-san-va-dang-cong-nhan-thang-11-1957-tai-matxcova-nga-3370</t>
+  </si>
+  <si>
+    <t>https://tse2.mm.bing.net/th/id/OIP.Zoxed5-nMtfNJ8Lp_NlMNgHaD4?r=0&amp;rs=1&amp;pid=ImgDetMain&amp;o=7&amp;rm=3</t>
   </si>
   <si>
     <t xml:space="preserve">18/12/1978 - 22/12/1978 </t>
@@ -548,6 +566,9 @@
 - Hội nghị khẳng định đường lối “giải phóng tư tưởng, thực sự cầu thị”, mở ra quá trình hiện đại hóa bốn lĩnh vực (nông nghiệp, công nghiệp, quốc phòng, khoa học – kỹ thuật).</t>
   </si>
   <si>
+    <t>http://vietnamese.china.org.cn/china_key_words/2022-10/12/content_78461979.htm</t>
+  </si>
+  <si>
     <t>Cuối thập niên 80 - đầu thập niên 90</t>
   </si>
   <si>
@@ -562,6 +583,9 @@
   </si>
   <si>
     <t>https://tapchilichsudang.vn/mot-so-yeu-to-tac-dong-den-su-hinh-thanh-duong-loi-xay-dung-chu-nghia-xa-hoi-o-mien-bac-1954-1975.html</t>
+  </si>
+  <si>
+    <t>https://th.bing.com/th/id/OIP.68mwPoMFrCywyIE5tr6j7AHaFl?w=312&amp;h=200&amp;c=10&amp;o=6&amp;pid=genserp&amp;rm=2</t>
   </si>
   <si>
     <t>08/11/2002 - 14/11/2002</t>
@@ -588,6 +612,9 @@
   <si>
     <t>- Đại hội XIX xác lập “Tư tưởng về chủ nghĩa xã hội đặc sắc Trung Quốc trong thời đại mới” của Tập Cận Bình, đưa tư tưởng này vào Cương lĩnh Đảng, khẳng định bước phát triển mới của mô hình XHCN mang đặc sắc Trung Quốc.
 - Đại hội đề ra mục tiêu đến giữa thế kỷ XXI xây dựng Trung Quốc trở thành nước xã hội chủ nghĩa hiện đại toàn diện, đồng thời nhấn mạnh vai trò lãnh đạo toàn diện của Đảng trong mọi lĩnh vực</t>
+  </si>
+  <si>
+    <t>https://baotintuc.vn/phan-tichnhan-dinh/dai-hoi-xix-cua-dang-cong-san-trung-quoc-diem-khoi-dau-lich-su-moi-cua-trung-quoc-20171021102418925.htm</t>
   </si>
   <si>
     <t>Các mốc thời gian quan trọng tại Việt Nam (Linh)</t>
@@ -732,7 +759,7 @@
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="166" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -750,6 +777,14 @@
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
     </font>
     <font>
       <u/>
@@ -792,10 +827,6 @@
     <font>
       <u/>
       <color rgb="FF1155CC"/>
-    </font>
-    <font>
-      <u/>
-      <color rgb="FF0000FF"/>
     </font>
     <font>
       <color theme="1"/>
@@ -1068,11 +1099,11 @@
     <xf borderId="8" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="9" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="8" fillId="0" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="8" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="8" fillId="0" fontId="3" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -1083,10 +1114,10 @@
     <xf borderId="11" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="11" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="11" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="12" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="12" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="12" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1101,22 +1132,22 @@
     <xf borderId="13" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="14" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="14" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="14" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="15" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="15" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="14" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="14" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
@@ -1125,29 +1156,26 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="8" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="9" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="8" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="8" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="8" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="8" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="8" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="8" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="8" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="8" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="8" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="8" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -1155,19 +1183,19 @@
     <xf borderId="14" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="14" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="14" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="14" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="14" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="8" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="8" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="14" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="15" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="15" fillId="0" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="15" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1176,7 +1204,10 @@
     <xf borderId="11" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="12" fillId="0" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="11" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="12" fillId="0" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1197,7 +1228,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Duong Van Hiep (K18 HL)" id="{d5a0bdcb-862f-4c62-a9b9-47379194e2b6}" providerId="google-sheets"/>
+  <x18tc:person displayName="Duong Van Hiep (K18 HL)" id="{b7122f3d-6d7f-489c-8a94-a8b19d646f01}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -1397,25 +1428,25 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="B31" dT="2026-07-01T02:47:28.00" personId="{d5a0bdcb-862f-4c62-a9b9-47379194e2b6}" id="{16ff7efc-bb06-4ebf-bbdf-5f8120576e3d}" done="1">
+  <x18tc:threadedComment ref="B31" dT="2026-07-01T02:47:28.00" personId="{b7122f3d-6d7f-489c-8a94-a8b19d646f01}" id="{da276ba1-998a-4cb2-a067-37f7d629c1c0}" done="1">
     <x18tc:text xml:space="preserve">chỗ nào mà lấy được ngày tháng bắt đầu kết thúc thì add vào nhé, đừng chỉ dừng ở mỗi năm</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="B31" dT="2026-07-01T02:57:50.00" personId="{d5a0bdcb-862f-4c62-a9b9-47379194e2b6}" id="{b5580a71-4059-4369-a342-5304095f5534}" parentId="{16ff7efc-bb06-4ebf-bbdf-5f8120576e3d}">
+  <x18tc:threadedComment ref="B31" dT="2026-07-01T02:57:50.00" personId="{b7122f3d-6d7f-489c-8a94-a8b19d646f01}" id="{f5492293-4405-4cce-97ab-2691746d6b41}" parentId="{da276ba1-998a-4cb2-a067-37f7d629c1c0}">
     <x18tc:text xml:space="preserve">thêm ngày thành lập đảng</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="A1" dT="2026-07-01T02:44:44.00" personId="{d5a0bdcb-862f-4c62-a9b9-47379194e2b6}" id="{3e40ec33-6cf3-4a33-afbb-39168adff873}" done="0">
+  <x18tc:threadedComment ref="A1" dT="2026-07-01T02:44:44.00" personId="{b7122f3d-6d7f-489c-8a94-a8b19d646f01}" id="{ed0e8a67-ea1c-430f-a164-aff19c26a351}" done="0">
     <x18tc:text xml:space="preserve">tìm cách thêm sự kiện và tách nhỏ hơn ra</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="A1" dT="2026-07-01T02:48:13.00" personId="{d5a0bdcb-862f-4c62-a9b9-47379194e2b6}" id="{6eeaa77a-379b-41f4-acd8-c5a0a98fc9b8}" parentId="{3e40ec33-6cf3-4a33-afbb-39168adff873}">
+  <x18tc:threadedComment ref="A1" dT="2026-07-01T02:48:13.00" personId="{b7122f3d-6d7f-489c-8a94-a8b19d646f01}" id="{cf1ae5a9-6c4b-4ff6-9ee3-5cd257fa8b74}" parentId="{ed0e8a67-ea1c-430f-a164-aff19c26a351}">
     <x18tc:text xml:space="preserve">chỗ nào mà lấy được ngày tháng bắt đầu kết thúc thì add vào nhé, đừng chỉ dừng ở mỗi năm</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="A21" dT="2026-07-01T02:46:49.00" personId="{d5a0bdcb-862f-4c62-a9b9-47379194e2b6}" id="{c996986f-a217-4480-9d9a-df812f454965}" done="1">
+  <x18tc:threadedComment ref="A21" dT="2026-07-01T02:46:49.00" personId="{b7122f3d-6d7f-489c-8a94-a8b19d646f01}" id="{05187ace-a827-4e19-a48d-f90aa28b5106}" done="1">
     <x18tc:text xml:space="preserve">phần này thấy có nhiều hội nghị, ngày, mình tìm thông tin về ngày tháng bắt đầu  kết thúc hội nghị nhé, thay vì chỉ dừng ở năm</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="B22" dT="2026-07-01T02:48:26.00" personId="{d5a0bdcb-862f-4c62-a9b9-47379194e2b6}" id="{de50ee63-2068-45ae-a900-546a2f628472}" done="0">
+  <x18tc:threadedComment ref="B22" dT="2026-07-01T02:48:26.00" personId="{b7122f3d-6d7f-489c-8a94-a8b19d646f01}" id="{4ee14459-0c2c-4c6e-95a6-49dd0ac33994}" done="0">
     <x18tc:text xml:space="preserve">phần này thấy có nhiều hội nghị, ngày, mình tìm thông tin về ngày tháng bắt đầu kết thúc hội nghị nhé, thay vì chỉ dừng ở năm</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="B3" dT="2026-07-01T02:48:03.00" personId="{d5a0bdcb-862f-4c62-a9b9-47379194e2b6}" id="{a36b1086-4032-47ad-bcee-8aaf3679ff8f}" done="0">
+  <x18tc:threadedComment ref="B3" dT="2026-07-01T02:48:03.00" personId="{b7122f3d-6d7f-489c-8a94-a8b19d646f01}" id="{4cb305d8-e3a5-4c11-9396-5e2500af0dcf}" done="0">
     <x18tc:text xml:space="preserve">chỗ nào mà lấy được ngày tháng bắt đầu kết thúc thì add vào nhé, đừng chỉ dừng ở mỗi năm</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -1425,6 +1456,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
@@ -1579,7 +1611,7 @@
       <c r="G4" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="13" t="s">
+      <c r="H4" s="17" t="s">
         <v>23</v>
       </c>
       <c r="I4" s="14"/>
@@ -1622,7 +1654,7 @@
       <c r="G5" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="H5" s="13" t="s">
+      <c r="H5" s="17" t="s">
         <v>30</v>
       </c>
       <c r="I5" s="14"/>
@@ -1690,7 +1722,7 @@
     </row>
     <row r="7">
       <c r="A7" s="10"/>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="18" t="s">
         <v>38</v>
       </c>
       <c r="C7" s="11" t="s">
@@ -1705,9 +1737,11 @@
       <c r="F7" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="G7" s="18"/>
+      <c r="G7" s="16" t="s">
+        <v>43</v>
+      </c>
       <c r="H7" s="13" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="I7" s="14"/>
       <c r="J7" s="9"/>
@@ -1732,25 +1766,25 @@
     <row r="8">
       <c r="A8" s="10"/>
       <c r="B8" s="11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H8" s="13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I8" s="14"/>
       <c r="J8" s="9"/>
@@ -1775,25 +1809,25 @@
     <row r="9">
       <c r="A9" s="10"/>
       <c r="B9" s="19" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I9" s="14"/>
       <c r="J9" s="9"/>
@@ -1818,23 +1852,25 @@
     <row r="10">
       <c r="A10" s="10"/>
       <c r="B10" s="19" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
-      <c r="G10" s="18"/>
+      <c r="G10" s="16" t="s">
+        <v>63</v>
+      </c>
       <c r="H10" s="13" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I10" s="14"/>
       <c r="J10" s="9"/>
@@ -1859,25 +1895,25 @@
     <row r="11">
       <c r="A11" s="10"/>
       <c r="B11" s="11" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I11" s="14"/>
       <c r="J11" s="9"/>
@@ -1902,23 +1938,25 @@
     <row r="12">
       <c r="A12" s="10"/>
       <c r="B12" s="11" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
-      <c r="G12" s="18"/>
+      <c r="G12" s="16" t="s">
+        <v>77</v>
+      </c>
       <c r="H12" s="13" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="I12" s="14"/>
       <c r="J12" s="9"/>
@@ -1943,23 +1981,25 @@
     <row r="13">
       <c r="A13" s="20"/>
       <c r="B13" s="21" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="F13" s="21" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
-      <c r="G13" s="22"/>
+      <c r="G13" s="22" t="s">
+        <v>84</v>
+      </c>
       <c r="H13" s="23" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="I13" s="24"/>
       <c r="J13" s="9"/>
@@ -1983,7 +2023,7 @@
     </row>
     <row r="14">
       <c r="A14" s="5" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -2015,28 +2055,28 @@
     <row r="15">
       <c r="A15" s="10"/>
       <c r="B15" s="11" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="H15" s="13" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="I15" s="13" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="J15" s="9"/>
       <c r="K15" s="9"/>
@@ -2060,28 +2100,28 @@
     <row r="16">
       <c r="A16" s="10"/>
       <c r="B16" s="11" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C16" s="26" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="F16" s="25" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="G16" s="12" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="I16" s="13" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="J16" s="9"/>
       <c r="K16" s="9"/>
@@ -2105,28 +2145,28 @@
     <row r="17">
       <c r="A17" s="27"/>
       <c r="B17" s="28" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D17" s="29" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="E17" s="25" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="F17" s="25" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="G17" s="30" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="H17" s="31" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="I17" s="31" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="J17" s="9"/>
       <c r="K17" s="9"/>
@@ -2150,28 +2190,28 @@
     <row r="18">
       <c r="A18" s="27"/>
       <c r="B18" s="25" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C18" s="32" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D18" s="29" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="E18" s="25" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="F18" s="25" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="G18" s="33" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="H18" s="31" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="I18" s="31" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="J18" s="9"/>
       <c r="K18" s="9"/>
@@ -2198,25 +2238,25 @@
         <v>8400.0</v>
       </c>
       <c r="C19" s="32" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D19" s="29" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="E19" s="25" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="F19" s="25" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="G19" s="33" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="H19" s="31" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="I19" s="31" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="J19" s="9"/>
       <c r="K19" s="9"/>
@@ -2243,25 +2283,25 @@
         <v>8787.0</v>
       </c>
       <c r="C20" s="36" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D20" s="29" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="E20" s="25" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="F20" s="25" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="G20" s="33" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="I20" s="31" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="J20" s="9"/>
       <c r="K20" s="9"/>
@@ -2284,7 +2324,7 @@
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
@@ -2316,28 +2356,28 @@
     <row r="22">
       <c r="A22" s="10"/>
       <c r="B22" s="11" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="G22" s="37" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
-      <c r="H22" s="38" t="s">
-        <v>128</v>
+      <c r="H22" s="17" t="s">
+        <v>132</v>
       </c>
-      <c r="I22" s="38" t="s">
-        <v>129</v>
+      <c r="I22" s="17" t="s">
+        <v>133</v>
       </c>
       <c r="J22" s="9"/>
       <c r="K22" s="9"/>
@@ -2361,25 +2401,29 @@
     <row r="23">
       <c r="A23" s="10"/>
       <c r="B23" s="11" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
-      <c r="G23" s="16" t="s">
-        <v>135</v>
+      <c r="G23" s="12" t="s">
+        <v>139</v>
       </c>
-      <c r="H23" s="14"/>
-      <c r="I23" s="14"/>
+      <c r="H23" s="13" t="s">
+        <v>140</v>
+      </c>
+      <c r="I23" s="13" t="s">
+        <v>139</v>
+      </c>
       <c r="J23" s="9"/>
       <c r="K23" s="9"/>
       <c r="L23" s="9"/>
@@ -2402,25 +2446,25 @@
     <row r="24">
       <c r="A24" s="10"/>
       <c r="B24" s="11" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
-      <c r="F24" s="39" t="s">
-        <v>139</v>
+      <c r="F24" s="38" t="s">
+        <v>144</v>
       </c>
       <c r="G24" s="12" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
-      <c r="H24" s="38" t="s">
-        <v>141</v>
+      <c r="H24" s="17" t="s">
+        <v>146</v>
       </c>
       <c r="I24" s="14"/>
       <c r="J24" s="9"/>
@@ -2445,24 +2489,26 @@
     <row r="25">
       <c r="A25" s="10"/>
       <c r="B25" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="C25" s="11" t="s">
         <v>142</v>
       </c>
-      <c r="C25" s="11" t="s">
-        <v>137</v>
-      </c>
       <c r="D25" s="11" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="G25" s="12" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
-      <c r="H25" s="14"/>
+      <c r="H25" s="17" t="s">
+        <v>151</v>
+      </c>
       <c r="I25" s="14"/>
       <c r="J25" s="9"/>
       <c r="K25" s="9"/>
@@ -2486,21 +2532,23 @@
     <row r="26">
       <c r="A26" s="10"/>
       <c r="B26" s="11" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
-      <c r="G26" s="18"/>
+      <c r="G26" s="12" t="s">
+        <v>157</v>
+      </c>
       <c r="H26" s="14"/>
       <c r="I26" s="14"/>
       <c r="J26" s="9"/>
@@ -2525,24 +2573,26 @@
     <row r="27">
       <c r="A27" s="10"/>
       <c r="B27" s="11" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="G27" s="16" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
-      <c r="H27" s="14"/>
+      <c r="H27" s="17" t="s">
+        <v>163</v>
+      </c>
       <c r="I27" s="14"/>
       <c r="J27" s="9"/>
       <c r="K27" s="9"/>
@@ -2566,21 +2616,23 @@
     <row r="28">
       <c r="A28" s="10"/>
       <c r="B28" s="11" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
-      <c r="F28" s="39" t="s">
-        <v>159</v>
+      <c r="F28" s="38" t="s">
+        <v>167</v>
       </c>
-      <c r="G28" s="40"/>
+      <c r="G28" s="12" t="s">
+        <v>140</v>
+      </c>
       <c r="H28" s="14"/>
       <c r="I28" s="14"/>
       <c r="J28" s="9"/>
@@ -2605,21 +2657,23 @@
     <row r="29">
       <c r="A29" s="20"/>
       <c r="B29" s="21" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="D29" s="21" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="E29" s="21" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="F29" s="21" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
-      <c r="G29" s="22"/>
+      <c r="G29" s="22" t="s">
+        <v>172</v>
+      </c>
       <c r="H29" s="24"/>
       <c r="I29" s="24"/>
       <c r="J29" s="9"/>
@@ -2643,7 +2697,7 @@
     </row>
     <row r="30">
       <c r="A30" s="5" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="B30" s="6"/>
       <c r="C30" s="6"/>
@@ -2675,25 +2729,25 @@
     <row r="31">
       <c r="A31" s="10"/>
       <c r="B31" s="11" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
-      <c r="C31" s="41" t="s">
-        <v>166</v>
+      <c r="C31" s="39" t="s">
+        <v>175</v>
       </c>
-      <c r="D31" s="42" t="s">
-        <v>167</v>
+      <c r="D31" s="40" t="s">
+        <v>176</v>
       </c>
-      <c r="E31" s="43" t="s">
-        <v>168</v>
+      <c r="E31" s="41" t="s">
+        <v>177</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="G31" s="12" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
-      <c r="H31" s="38" t="s">
-        <v>171</v>
+      <c r="H31" s="17" t="s">
+        <v>180</v>
       </c>
       <c r="I31" s="14"/>
       <c r="J31" s="9"/>
@@ -2718,25 +2772,25 @@
     <row r="32">
       <c r="A32" s="10"/>
       <c r="B32" s="11" t="s">
-        <v>172</v>
+        <v>181</v>
       </c>
-      <c r="C32" s="41" t="s">
-        <v>173</v>
+      <c r="C32" s="39" t="s">
+        <v>182</v>
       </c>
-      <c r="D32" s="42" t="s">
-        <v>174</v>
+      <c r="D32" s="40" t="s">
+        <v>183</v>
       </c>
-      <c r="E32" s="43" t="s">
-        <v>175</v>
+      <c r="E32" s="41" t="s">
+        <v>184</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="G32" s="12" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
-      <c r="H32" s="38" t="s">
-        <v>178</v>
+      <c r="H32" s="17" t="s">
+        <v>187</v>
       </c>
       <c r="I32" s="14"/>
       <c r="J32" s="9"/>
@@ -2763,19 +2817,19 @@
       <c r="B33" s="19">
         <v>16808.0</v>
       </c>
-      <c r="C33" s="41" t="s">
-        <v>179</v>
+      <c r="C33" s="39" t="s">
+        <v>188</v>
       </c>
-      <c r="D33" s="43"/>
-      <c r="E33" s="43" t="s">
-        <v>180</v>
+      <c r="D33" s="41"/>
+      <c r="E33" s="41" t="s">
+        <v>189</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
-      <c r="G33" s="18"/>
-      <c r="H33" s="38" t="s">
-        <v>182</v>
+      <c r="G33" s="42"/>
+      <c r="H33" s="17" t="s">
+        <v>191</v>
       </c>
       <c r="I33" s="14"/>
       <c r="J33" s="9"/>
@@ -2802,21 +2856,21 @@
       <c r="B34" s="19">
         <v>27943.0</v>
       </c>
-      <c r="C34" s="41" t="s">
-        <v>183</v>
+      <c r="C34" s="39" t="s">
+        <v>192</v>
       </c>
-      <c r="D34" s="42" t="s">
-        <v>184</v>
+      <c r="D34" s="40" t="s">
+        <v>193</v>
       </c>
-      <c r="E34" s="43" t="s">
-        <v>185</v>
+      <c r="E34" s="41" t="s">
+        <v>194</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
-      <c r="G34" s="18"/>
-      <c r="H34" s="38" t="s">
-        <v>187</v>
+      <c r="G34" s="42"/>
+      <c r="H34" s="17" t="s">
+        <v>196</v>
       </c>
       <c r="I34" s="14"/>
       <c r="J34" s="9"/>
@@ -2840,24 +2894,24 @@
     </row>
     <row r="35">
       <c r="A35" s="10"/>
-      <c r="B35" s="44" t="s">
-        <v>188</v>
+      <c r="B35" s="43" t="s">
+        <v>197</v>
       </c>
-      <c r="C35" s="41" t="s">
-        <v>189</v>
+      <c r="C35" s="39" t="s">
+        <v>198</v>
       </c>
-      <c r="D35" s="42" t="s">
-        <v>184</v>
+      <c r="D35" s="40" t="s">
+        <v>193</v>
       </c>
-      <c r="E35" s="42" t="s">
-        <v>190</v>
+      <c r="E35" s="40" t="s">
+        <v>199</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
-      <c r="G35" s="18"/>
-      <c r="H35" s="38" t="s">
-        <v>192</v>
+      <c r="G35" s="42"/>
+      <c r="H35" s="17" t="s">
+        <v>201</v>
       </c>
       <c r="I35" s="14"/>
       <c r="J35" s="9"/>
@@ -2881,26 +2935,26 @@
     </row>
     <row r="36">
       <c r="A36" s="27"/>
-      <c r="B36" s="45" t="s">
+      <c r="B36" s="44" t="s">
+        <v>202</v>
+      </c>
+      <c r="C36" s="45" t="s">
+        <v>203</v>
+      </c>
+      <c r="D36" s="46" t="s">
         <v>193</v>
       </c>
-      <c r="C36" s="46" t="s">
-        <v>194</v>
-      </c>
-      <c r="D36" s="47" t="s">
-        <v>184</v>
-      </c>
-      <c r="E36" s="48" t="s">
-        <v>195</v>
+      <c r="E36" s="47" t="s">
+        <v>204</v>
       </c>
       <c r="F36" s="29" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
-      <c r="G36" s="49"/>
-      <c r="H36" s="50" t="s">
-        <v>197</v>
+      <c r="G36" s="48"/>
+      <c r="H36" s="49" t="s">
+        <v>206</v>
       </c>
-      <c r="I36" s="51"/>
+      <c r="I36" s="50"/>
       <c r="J36" s="9"/>
       <c r="K36" s="9"/>
       <c r="L36" s="9"/>
@@ -2922,28 +2976,28 @@
     </row>
     <row r="37">
       <c r="A37" s="27"/>
-      <c r="B37" s="45" t="s">
+      <c r="B37" s="44" t="s">
+        <v>207</v>
+      </c>
+      <c r="C37" s="29" t="s">
         <v>198</v>
       </c>
-      <c r="C37" s="29" t="s">
-        <v>189</v>
-      </c>
       <c r="D37" s="29" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="E37" s="29" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="F37" s="29" t="s">
-        <v>200</v>
+        <v>209</v>
       </c>
       <c r="G37" s="30" t="s">
-        <v>201</v>
+        <v>210</v>
       </c>
-      <c r="H37" s="50" t="s">
-        <v>202</v>
+      <c r="H37" s="49" t="s">
+        <v>211</v>
       </c>
-      <c r="I37" s="51"/>
+      <c r="I37" s="50"/>
       <c r="J37" s="9"/>
       <c r="K37" s="9"/>
       <c r="L37" s="9"/>
@@ -2965,24 +3019,24 @@
     </row>
     <row r="38">
       <c r="A38" s="20"/>
-      <c r="B38" s="52" t="s">
-        <v>203</v>
+      <c r="B38" s="51" t="s">
+        <v>212</v>
       </c>
       <c r="C38" s="21" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="D38" s="21" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="E38" s="21" t="s">
-        <v>204</v>
+        <v>213</v>
       </c>
       <c r="F38" s="21" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
-      <c r="G38" s="22"/>
+      <c r="G38" s="52"/>
       <c r="H38" s="53" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="I38" s="24"/>
       <c r="J38" s="9"/>
@@ -3007,7 +3061,7 @@
     <row r="39">
       <c r="A39" s="9"/>
       <c r="B39" s="32" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="C39" s="9"/>
       <c r="D39" s="9"/>
@@ -31500,56 +31554,70 @@
     <hyperlink r:id="rId9" ref="H5"/>
     <hyperlink r:id="rId10" ref="G6"/>
     <hyperlink r:id="rId11" ref="H6"/>
-    <hyperlink r:id="rId12" ref="H7"/>
-    <hyperlink r:id="rId13" ref="G8"/>
-    <hyperlink r:id="rId14" ref="H8"/>
-    <hyperlink r:id="rId15" ref="G9"/>
-    <hyperlink r:id="rId16" ref="H9"/>
-    <hyperlink r:id="rId17" ref="H10"/>
-    <hyperlink r:id="rId18" ref="G11"/>
-    <hyperlink r:id="rId19" ref="H11"/>
-    <hyperlink r:id="rId20" ref="H12"/>
-    <hyperlink r:id="rId21" ref="H13"/>
-    <hyperlink r:id="rId22" ref="G15"/>
-    <hyperlink r:id="rId23" location="/media/File:Lenin_book_1902.jpg" ref="H15"/>
-    <hyperlink r:id="rId24" ref="I15"/>
-    <hyperlink r:id="rId25" ref="G16"/>
-    <hyperlink r:id="rId26" location="gallery" ref="H16"/>
-    <hyperlink r:id="rId27" ref="I16"/>
-    <hyperlink r:id="rId28" ref="G17"/>
-    <hyperlink r:id="rId29" ref="H17"/>
-    <hyperlink r:id="rId30" ref="I17"/>
-    <hyperlink r:id="rId31" ref="G18"/>
-    <hyperlink r:id="rId32" ref="H18"/>
-    <hyperlink r:id="rId33" ref="I18"/>
-    <hyperlink r:id="rId34" ref="G19"/>
-    <hyperlink r:id="rId35" ref="H19"/>
-    <hyperlink r:id="rId36" ref="I19"/>
-    <hyperlink r:id="rId37" ref="C20"/>
-    <hyperlink r:id="rId38" ref="G20"/>
-    <hyperlink r:id="rId39" ref="H20"/>
-    <hyperlink r:id="rId40" ref="I20"/>
-    <hyperlink r:id="rId41" ref="G22"/>
-    <hyperlink r:id="rId42" ref="H22"/>
-    <hyperlink r:id="rId43" ref="I22"/>
-    <hyperlink r:id="rId44" ref="G23"/>
-    <hyperlink r:id="rId45" ref="G24"/>
-    <hyperlink r:id="rId46" ref="H24"/>
-    <hyperlink r:id="rId47" ref="G25"/>
-    <hyperlink r:id="rId48" ref="G27"/>
-    <hyperlink r:id="rId49" ref="G31"/>
-    <hyperlink r:id="rId50" ref="H31"/>
-    <hyperlink r:id="rId51" ref="G32"/>
-    <hyperlink r:id="rId52" ref="H32"/>
-    <hyperlink r:id="rId53" ref="H33"/>
-    <hyperlink r:id="rId54" ref="H34"/>
-    <hyperlink r:id="rId55" ref="H35"/>
-    <hyperlink r:id="rId56" ref="H36"/>
-    <hyperlink r:id="rId57" ref="G37"/>
-    <hyperlink r:id="rId58" ref="H37"/>
-    <hyperlink r:id="rId59" ref="H38"/>
+    <hyperlink r:id="rId12" ref="G7"/>
+    <hyperlink r:id="rId13" ref="H7"/>
+    <hyperlink r:id="rId14" ref="G8"/>
+    <hyperlink r:id="rId15" ref="H8"/>
+    <hyperlink r:id="rId16" ref="G9"/>
+    <hyperlink r:id="rId17" ref="H9"/>
+    <hyperlink r:id="rId18" ref="G10"/>
+    <hyperlink r:id="rId19" ref="H10"/>
+    <hyperlink r:id="rId20" ref="G11"/>
+    <hyperlink r:id="rId21" ref="H11"/>
+    <hyperlink r:id="rId22" ref="G12"/>
+    <hyperlink r:id="rId23" ref="H12"/>
+    <hyperlink r:id="rId24" ref="G13"/>
+    <hyperlink r:id="rId25" ref="H13"/>
+    <hyperlink r:id="rId26" ref="G15"/>
+    <hyperlink r:id="rId27" location="/media/File:Lenin_book_1902.jpg" ref="H15"/>
+    <hyperlink r:id="rId28" ref="I15"/>
+    <hyperlink r:id="rId29" ref="G16"/>
+    <hyperlink r:id="rId30" location="gallery" ref="H16"/>
+    <hyperlink r:id="rId31" ref="I16"/>
+    <hyperlink r:id="rId32" ref="G17"/>
+    <hyperlink r:id="rId33" ref="H17"/>
+    <hyperlink r:id="rId34" ref="I17"/>
+    <hyperlink r:id="rId35" ref="G18"/>
+    <hyperlink r:id="rId36" ref="H18"/>
+    <hyperlink r:id="rId37" ref="I18"/>
+    <hyperlink r:id="rId38" ref="G19"/>
+    <hyperlink r:id="rId39" ref="H19"/>
+    <hyperlink r:id="rId40" ref="I19"/>
+    <hyperlink r:id="rId41" ref="C20"/>
+    <hyperlink r:id="rId42" ref="G20"/>
+    <hyperlink r:id="rId43" ref="H20"/>
+    <hyperlink r:id="rId44" ref="I20"/>
+    <hyperlink r:id="rId45" ref="G22"/>
+    <hyperlink r:id="rId46" ref="H22"/>
+    <hyperlink r:id="rId47" ref="I22"/>
+    <hyperlink r:id="rId48" ref="G23"/>
+    <hyperlink r:id="rId49" ref="H23"/>
+    <hyperlink r:id="rId50" ref="I23"/>
+    <hyperlink r:id="rId51" ref="G24"/>
+    <hyperlink r:id="rId52" ref="H24"/>
+    <hyperlink r:id="rId53" ref="G25"/>
+    <hyperlink r:id="rId54" ref="H25"/>
+    <hyperlink r:id="rId55" ref="G26"/>
+    <hyperlink r:id="rId56" ref="G27"/>
+    <hyperlink r:id="rId57" ref="H27"/>
+    <hyperlink r:id="rId58" ref="G28"/>
+    <hyperlink r:id="rId59" ref="G29"/>
+    <hyperlink r:id="rId60" ref="G31"/>
+    <hyperlink r:id="rId61" ref="H31"/>
+    <hyperlink r:id="rId62" ref="G32"/>
+    <hyperlink r:id="rId63" ref="H32"/>
+    <hyperlink r:id="rId64" ref="H33"/>
+    <hyperlink r:id="rId65" ref="H34"/>
+    <hyperlink r:id="rId66" ref="H35"/>
+    <hyperlink r:id="rId67" ref="H36"/>
+    <hyperlink r:id="rId68" ref="G37"/>
+    <hyperlink r:id="rId69" ref="H37"/>
+    <hyperlink r:id="rId70" ref="H38"/>
   </hyperlinks>
-  <drawing r:id="rId60"/>
-  <legacyDrawing r:id="rId61"/>
+  <printOptions gridLines="1" horizontalCentered="1"/>
+  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageSetup fitToHeight="0" paperSize="9" cellComments="atEnd" orientation="landscape" pageOrder="overThenDown"/>
+  <drawing r:id="rId71"/>
+  <legacyDrawing r:id="rId72"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: replace Knowledge Panel with Q&A chatbot, revise content
- Add ChatPanel (Ctrl+K) backed by api/chat.ts serverless endpoint;
  chat history/pending state lives in useMuseumStore
- Remove KnowledgePanel, exclude /api from SPA rewrite in vercel.json
- Add .env.example and ignore .env* for OPENAI_API_KEY
- Content audit fixes via scripts/content-fixes (content.json, quiz,
  docs/content.xlsx, content-report)
- Simplify Vietnam room background (drop 200vh bamboo parallax)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/content.xlsx
+++ b/docs/content.xlsx
@@ -78,13 +78,13 @@
     <t>45.774272, 4.829994</t>
   </si>
   <si>
-    <t>Phong trào đấu tranh của giai cấp công nhân tại thành phố Lion, Pháp giương cao khẩu hiệu về kinh tế và chính trị,.</t>
+    <t>Phong trào đấu tranh của giai cấp công nhân tại thành phố Lyon, Pháp giương cao khẩu hiệu về kinh tế và chính trị.</t>
   </si>
   <si>
     <t>Đây là các cuộc đấu tranh lớn của thợ dệt lụa Lyon. Phong trào nêu yêu sách kinh tế về tiền công, điều kiện sống, đồng thời thể hiện bước phát triển về ý thức chính trị của giai cấp công nhân. Đây thường được xem là một trong những cuộc đấu tranh công nhân tiêu biểu đầu thế kỷ XIX.</t>
   </si>
   <si>
-    <t>https://www.gadagne-lyon.fr/sites/gadagne/files/medias/documents/2020-12/MHL-Gadagne_ThemedSheet_19th-TheCanutRevolts.pdf?utm_source=chatgpt.com</t>
+    <t>https://www.gadagne-lyon.fr/sites/gadagne/files/medias/documents/2020-12/MHL-Gadagne_ThemedSheet_19th-TheCanutRevolts.pdf</t>
   </si>
   <si>
     <t>https://upload.wikimedia.org/wikipedia/commons/4/45/Revolte_des_Canuts_-_Lyon_1831_-_1.jpg</t>
@@ -105,7 +105,7 @@
     <t>Phong trào Hiến chương là phong trào chính trị rộng lớn của giai cấp công nhân Anh, xuất hiện từ năm 1836 và hoạt động mạnh nhất trong giai đoạn 1838–1848. Mục tiêu là đòi quyền chính trị cho người lao động, tiêu biểu qua “Hiến chương Nhân dân”.</t>
   </si>
   <si>
-    <t>https://www.nationalarchives.gov.uk/education/resources/what-was-chartism/?utm_source=chatgpt.com</t>
+    <t>https://www.nationalarchives.gov.uk/education/resources/what-was-chartism/</t>
   </si>
   <si>
     <t>https://upload.wikimedia.org/wikipedia/commons/2/24/Chartist_meeting%2C_Kennington_Common.jpg</t>
@@ -126,7 +126,7 @@
     <t>Cuộc nổi dậy của thợ dệt Silesia nổ ra năm 1844, bắt đầu tại Peterswaldau, nay là Pieszyce, rồi lan sang các khu vực lân cận. Nguyên nhân chính là tiền công thấp, đời sống khó khăn và sự bóc lột của giới chủ/thầu trung gian.</t>
   </si>
   <si>
-    <t>https://www.deutschlandmuseum.de/en/history/calendar/1844-06-04-the-weavers-revolt/?utm_source=chatgpt.com</t>
+    <t>https://www.deutschlandmuseum.de/en/history/calendar/1844-06-04-the-weavers-revolt/</t>
   </si>
   <si>
     <t>https://upload.wikimedia.org/wikipedia/commons/9/9f/Carl_Wilhelm_H%C3%BCbner_-_The_Silesian_Weavers_-_Google_Art_Project.jpg</t>
@@ -148,13 +148,13 @@
     <t>Giai đoạn này Mác và Ăngghen chuyển từ lập trường dân chủ cách mạng sang lập trường cộng sản. Mác nghiên cứu sâu về triết học, chính trị và kinh tế; Ăngghen nghiên cứu thực tiễn đời sống giai cấp công nhân ở Anh. Năm 1844, hai ông bắt đầu hợp tác chặt chẽ tại Paris, tạo tiền đề cho sự hình thành CNXHKH.</t>
   </si>
   <si>
-    <t>https://thinhvuongvietnam.com/Content/ky-niem-202-nam-ngay-sinh-cmac-551818---552020-cmac-va-hanh-trinh-den-voi-chu-nghia-cong-san-31623?utm_source=chatgpt.com</t>
+    <t>https://thinhvuongvietnam.com/Content/ky-niem-202-nam-ngay-sinh-cmac-551818---552020-cmac-va-hanh-trinh-den-voi-chu-nghia-cong-san-31623</t>
   </si>
   <si>
     <t>https://upload.wikimedia.org/wikipedia/commons/7/79/Marx_and_Engels.jpg</t>
   </si>
   <si>
-    <t>2/1848</t>
+    <t>Tháng 2/1848</t>
   </si>
   <si>
     <t>46 Liverpool Street, Bishopsgate, London, Anh</t>
@@ -169,7 +169,7 @@
     <t>Tác phẩm do C. Mác và Ph. Ăngghen soạn thảo, được công bố lần đầu bằng tiếng Đức vào tháng 2/1848 tại London. Tác phẩm đánh dấu sự ra đời về mặt lý luận của chủ nghĩa xã hội khoa học.</t>
   </si>
   <si>
-    <t>https://tulieuvankien.dangcongsan.vn/ho-so-su-kien-nhan-chung/su-kien-va-nhan-chung/tuyen-ngon-dang-cong-san-thang-2-1848-3385?utm_source=chatgpt.com</t>
+    <t>https://tulieuvankien.dangcongsan.vn/ho-so-su-kien-nhan-chung/su-kien-va-nhan-chung/tuyen-ngon-dang-cong-san-thang-2-1848-3385</t>
   </si>
   <si>
     <t>https://upload.wikimedia.org/wikipedia/commons/thumb/8/86/Communist-manifesto.png/500px-Communist-manifesto.png?_=20251104221727</t>
@@ -184,13 +184,13 @@
     <t>48.8566, 2.3522</t>
   </si>
   <si>
-    <t>Các cuộc cách mạng dân chủ tư sản diễn ra tại các nước Tây Âu,.</t>
+    <t>Các cuộc cách mạng dân chủ tư sản diễn ra tại các nước Tây Âu.</t>
   </si>
   <si>
     <t>Cách mạng 1848 thường được gọi là “Mùa xuân của các dân tộc”, bắt đầu lan rộng ở châu Âu từ năm 1848, tiêu biểu tại Pháp, Đức, Áo, Ý. Trong học phần, mốc 1848–1852 có thể hiểu là giai đoạn diễn ra, thất bại và được Mác – Ăngghen tổng kết kinh nghiệm cách mạng.</t>
   </si>
   <si>
-    <t>https://www.history.com/a-year-in-history/1848?utm_source=chatgpt.com</t>
+    <t>https://www.history.com/a-year-in-history/1848</t>
   </si>
   <si>
     <t>https://upload.wikimedia.org/wikipedia/commons/thumb/2/26/Barricades_rue_Saint-Maur._Avant_l%27attaque%2C_25_juin_1848._Apr%C3%A8s_l%E2%80%99attaque%2C_26_juin_1848.jpg/960px-Barricades_rue_Saint-Maur._Avant_l%27attaque%2C_25_juin_1848._Apr%C3%A8s_l%E2%80%99attaque%2C_26_juin_1848.jpg?_=20230922071523</t>
@@ -211,7 +211,7 @@
     <t>Ngày 28/9/1864, Hội Liên hiệp Công nhân Quốc tế, thường gọi là Quốc tế I, được thành lập tại St Martin’s Hall, London. Tổ chức này góp phần liên kết phong trào công nhân quốc tế.</t>
   </si>
   <si>
-    <t>https://tulieuvankien.dangcongsan.vn/ho-so-su-kien-nhan-chung/phong-trao-cong-san-cong-nhan-quoc-te/quoc-te-cong-san/quoc-te-i-1864-1876-103?utm_source=chatgpt.com</t>
+    <t>https://tulieuvankien.dangcongsan.vn/ho-so-su-kien-nhan-chung/phong-trao-cong-san-cong-nhan-quoc-te/quoc-te-cong-san/quoc-te-i-1864-1876-103</t>
   </si>
   <si>
     <t>14/09/1867</t>
@@ -229,7 +229,7 @@
     <t>Tập I của bộ Tư bản do C. Mác viết, xuất bản lần đầu bằng tiếng Đức tại Hamburg bởi nhà xuất bản Otto Meissner năm 1867. Đây là tác phẩm phân tích sâu sắc phương thức sản xuất tư bản chủ nghĩa.</t>
   </si>
   <si>
-    <t>https://germanhistorydocs.org/en/forging-an-empire-bismarckian-germany-1866-1890/karl-marx-capital-das-kapital-cover-of-the-1st-edition-1867?utm_source=chatgpt.com</t>
+    <t>https://germanhistorydocs.org/en/forging-an-empire-bismarckian-germany-1866-1890/karl-marx-capital-das-kapital-cover-of-the-1st-edition-1867</t>
   </si>
   <si>
     <t>https://upload.wikimedia.org/wikipedia/commons/d/da/Marx_-_Das_Kapital_-_1867_-_DHM.JPG</t>
@@ -244,7 +244,7 @@
     <t>48.856373, 2.353016</t>
   </si>
   <si>
-    <t>Sự kiện Công xã Pari tại Pháp tạo ra hình thái nhà nước mới của giai cấp công nhân,,.</t>
+    <t>Sự kiện Công xã Pari tại Pháp tạo ra hình thái nhà nước mới của giai cấp công nhân.</t>
   </si>
   <si>
     <t>Công xã Paris tồn tại từ 18/3 đến 28/5/1871. Đây là chính quyền cách mạng của nhân dân lao động Paris, thường được xem là hình thức nhà nước mới đầu tiên của giai cấp công nhân.</t>
@@ -286,13 +286,13 @@
     <t>51.3397, 12.3731</t>
   </si>
   <si>
-    <t>Ph. Ăngghen viết tác phẩm "Chống Đuyrinh",.</t>
+    <t>Ph. Ăngghen viết tác phẩm "Chống Đuyrinh".</t>
   </si>
   <si>
     <t>“Chống Đuyrinh” do Ph. Ăngghen viết trong giai đoạn 1876–1878, đăng nhiều kỳ trên báo Vorwärts và xuất bản thành sách tại Leipzig năm 1878. Tác phẩm trình bày có hệ thống nhiều nội dung cơ bản của chủ nghĩa Mác.</t>
   </si>
   <si>
-    <t>https://luatminhkhue.vn/gioi-thieu-khai-quat-tac-pham-chong-duyrinh-cua-ph-angghen.aspx</t>
+    <t>https://www.quanlynhanuoc.vn/2024/07/25/gia-tri-tu-tuong-ph-angghen-ve-chu-nghia-duy-vat-bien-chung-trong-tac-pham-chong-duyrinh/</t>
   </si>
   <si>
     <t>https://upload.wikimedia.org/wikipedia/commons/thumb/3/3a/Anti_Duhring_cover.jpg/500px-Anti_Duhring_cover.jpg?_=20260205183536</t>
@@ -322,7 +322,7 @@
     <t>https://en.wikipedia.org/wiki/What_Is_to_Be_Done%3F#/media/File:Lenin_book_1902.jpg</t>
   </si>
   <si>
-    <t xml:space="preserve"> 6/11/1917-7/11/1917</t>
+    <t>06/11/1917 - 07/11/1917</t>
   </si>
   <si>
     <t>Petrograd (nay là thành phố Saint Petersburg), Nga.</t>
@@ -331,7 +331,7 @@
     <t>59.91811876813978, 30.308775637783157</t>
   </si>
   <si>
-    <t>Cách mạng Tháng Mười Nga thành công, dẫn đến sự ra đời của Nhà nước Xôviết - nhà nước XHCN đầu tiên trên thế giới tại Nga,,.</t>
+    <t>Cách mạng Tháng Mười Nga thành công, dẫn đến sự ra đời của Nhà nước Xôviết - nhà nước XHCN đầu tiên trên thế giới tại Nga.</t>
   </si>
   <si>
     <t>Dưới sự lãnh đạo trực tiếp của Lênin và Đảng Bolshevik, lực lượng công nhân, binh lính và thủy thủ đã lật đổ Chính phủ lâm thời tư sản, giành chính quyền về tay các Xô viết. Đây là cuộc cách mạng vô sản đầu tiên trên thế giới giành thắng lợi.</t>
@@ -343,7 +343,7 @@
     <t>https://www.baoquankhu7.vn/cach-mang-thang-muoi-nga-chi-ra-con-duong-giai-phong-dan-toc-viet-nam--1378944605-0041678s34010gs#gallery</t>
   </si>
   <si>
-    <t>2/3/1919 - 6/3/1919</t>
+    <t>02/03/1919 - 06/03/1919</t>
   </si>
   <si>
     <t>Mát-xcơ-va (Moscow), Nga</t>
@@ -367,7 +367,7 @@
     <t>https://special.vietnamplus.vn/su-ra-doi-cua-quoc-te-cong-san-quoc-te-iii-vao-thang-3-1919-da-thuc-day-su-phat-trien-manh-me-phong-trao-cong-san-va-cong-nhan-quoc-te-doi-voi-viet-nam-quoc-te-cong-san-co-vai-tro-quan-trong-tro/</t>
   </si>
   <si>
-    <t>tháng 3 năm 1921</t>
+    <t>Tháng 3/1921</t>
   </si>
   <si>
     <t>V.I. Lênin khởi xướng và lãnh đạo thực hiện "Chính sách Kinh tế mới" (NEP).</t>
@@ -397,13 +397,7 @@
     <t>https://vpdf.org.vn/tin-tuc-su-kien/chinh-tri-xa-hoi/su-ra-doi-cua-lien-bang-xo-viet-mot-the-ky-nhin-lai.html</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u/>
-        <color rgb="FF1155CC"/>
-      </rPr>
-      <t>Gorki Leninskie, Nga</t>
-    </r>
+    <t>Gorki (nay là Gorki Leninskiye), ngoại ô Mátxcơva, Nga</t>
   </si>
   <si>
     <t>55.50858968707844, 37.77730781373274</t>
@@ -424,26 +418,25 @@
     <t>Giai đoạn từ sau khi V.I. Lênin qua đời đến nay - Tuấn Anh</t>
   </si>
   <si>
-    <t>Ngày 1/7/1921</t>
+    <t>01/07/1921</t>
   </si>
   <si>
     <t xml:space="preserve">Thượng Hải (Trung Quốc), sau đó phiên họp hoàn tất trên một 
-con thuyền ở Hồ Nam, Gia Hưng, tỉnh Chiết Giang</t>
+con thuyền ở Nam Hồ, Gia Hưng, tỉnh Chiết Giang</t>
   </si>
   <si>
     <t xml:space="preserve">Thượng Hải - 31.2415424510595, 121.47258398699829
-Hồ Nam - 30.758488630622896, 120.75395555515016</t>
+Nam Hồ, Gia Hưng, Chiết Giang - 30.758488630622896, 120.75395555515016</t>
   </si>
   <si>
     <t>Đảng Cộng sản Trung Quốc được thành lập tại Trung Quốc.</t>
   </si>
   <si>
-    <t xml:space="preserve">-Đại hội lần thứ nhất của CPC họp với 13 đại biểu, đại diện cho khoảng 50 đảng viên, đánh dấu sự ra đời của chính đảng mác-xít ở Trung Quốc
--Sau này Đảng Cộng sản Trung Quốc chính thức lấy ngày 1/7/1921 làm ngày thành lập để kỷ niệm thường niên.</t>
+    <t xml:space="preserve">- Đại hội lần thứ nhất của CPC họp với 13 đại biểu, đại diện cho khoảng 50 đảng viên, đánh dấu sự ra đời của chính đảng mác-xít ở Trung Quốc.
+- Sau này Đảng Cộng sản Trung Quốc chính thức lấy ngày 1/7/1921 làm ngày thành lập để kỷ niệm thường niên.</t>
   </si>
   <si>
-    <t xml:space="preserve">http://vietnamese.china.org.cn/china_key_words/2022-10/12/content_78462169.htm
-https://vi.wikipedia.org/wiki/%C4%90%E1%BA%A3ng_C%E1%BB%99ng_s%E1%BA%A3n_Trung_Qu%E1%BB%91c</t>
+    <t>https://tulieuvankien.dangcongsan.vn/ho-so-su-kien-nhan-chung/phong-trao-cong-san-cong-nhan-quoc-te/cac-dang-cong-san-cong-nhan/dang-cong-san-trung-quoc-3267</t>
   </si>
   <si>
     <t>https://upload.wikimedia.org/wikipedia/commons/8/85/Mao_Proclaiming_New_China.JPG</t>
@@ -466,8 +459,8 @@
     <t>Chiến tranh thế giới thứ hai diễn ra, sau đó hệ thống xã hội chủ nghĩa thế giới hình thành.</t>
   </si>
   <si>
-    <t xml:space="preserve">-Sau Chiến tranh thế giới thứ hai, Liên Xô mở rộng ảnh hưởng sang Đông Âu, góp phần hình thành hệ thống các nước xã hội chủ nghĩa ở châu Âu (Ba Lan, Tiệp Khắc, Đông Đức, Hungary, Romania, Bulgaria, Albania, v.v.
--Thắng lợi của Hồng quân Liên Xô và phong trào giải phóng dân tộc thúc đẩy sự mở rộng của trật tự xã hội chủ nghĩa trên phạm vi toàn cầu, tạo tiền đề cho sự đối lập giữa hai hệ thống: tư bản chủ nghĩa và xã hội chủ nghĩa.</t>
+    <t xml:space="preserve">- Sau Chiến tranh thế giới thứ hai, Liên Xô mở rộng ảnh hưởng sang Đông Âu, góp phần hình thành hệ thống các nước xã hội chủ nghĩa ở châu Âu (Ba Lan, Tiệp Khắc, Đông Đức, Hungary, Romania, Bulgaria, Albania, v.v.).
+- Thắng lợi của Hồng quân Liên Xô và phong trào giải phóng dân tộc thúc đẩy sự mở rộng của trật tự xã hội chủ nghĩa trên phạm vi toàn cầu, tạo tiền đề cho sự đối lập giữa hai hệ thống: tư bản chủ nghĩa và xã hội chủ nghĩa.</t>
   </si>
   <si>
     <t>https://vi.wikipedia.org/wiki/Chi%E1%BA%BFn_tranh_th%E1%BA%BF_gi%E1%BB%9Bi_th%E1%BB%A9_hai</t>
@@ -488,28 +481,27 @@
     <t>Hội nghị đại biểu các Đảng Cộng sản và công nhân quốc tế họp tại Mátxcơva, Nga thông qua 9 quy luật chung của công cuộc cải tạo XHCN.</t>
   </si>
   <si>
-    <t xml:space="preserve">- Hội nghị đại biểu các Đảng Cộng sản và công nhân quốc tế họp tại Moskva tháng 11/1957, tổng kết thực tiễn xây dựng chủ nghĩa xã hội và thông qua 9 quy luật chung của công cuộc cải tạo xã hội chủ nghĩa
-- Văn kiện từ hội nghị này trở thành cơ sở quan trọng để các Đảng Mác – Lênin vận dụng trong đường lối xây dựng mô hình xã hội chủ nghĩa ở các nước xã hội chủ nghĩa, trong đó có Việt Nam</t>
+    <t xml:space="preserve">- Hội nghị đại biểu các Đảng Cộng sản và công nhân quốc tế họp tại Moskva tháng 11/1957, tổng kết thực tiễn xây dựng chủ nghĩa xã hội và thông qua 9 quy luật chung của công cuộc cải tạo xã hội chủ nghĩa.
+- Văn kiện từ hội nghị này trở thành cơ sở quan trọng để các Đảng Mác – Lênin vận dụng trong đường lối xây dựng mô hình xã hội chủ nghĩa ở các nước xã hội chủ nghĩa, trong đó có Việt Nam.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://tulieuvankien.dangcongsan.vn/ho-so-su-kien-nhan-chung/su-kien-va-nhan-chung?page=1
-</t>
+    <t>https://tulieuvankien.dangcongsan.vn/ho-so-su-kien-nhan-chung/su-kien-va-nhan-chung/hoi-nghi-dai-bieu-cac-dang-cong-san-va-dang-cong-nhan-thang-11-1957-tai-matxcova-nga-3370</t>
   </si>
   <si>
     <t>https://hochiminh-image.nhandan.vn/t460/Uploaded/tgshzb/2022_05_06/17-12-1960_phong_trao_cong_san_va_cong_nhan___.jpg</t>
   </si>
   <si>
-    <t>Tháng 1/1960</t>
+    <t>Tháng 11/1960</t>
   </si>
   <si>
     <t>Hội nghị đại biểu của 81 Đảng Cộng sản và công nhân quốc tế họp tại Mátxcơva, Nga phân tích tình hình quốc tế và đưa ra khái niệm về "thời đại hiện nay".</t>
   </si>
   <si>
-    <t xml:space="preserve">- Hội nghị đại biểu của 81 Đảng Cộng sản và Đảng Công nhân quốc tế họp ở Moskva tháng 01/1960, phân tích tình hình quốc tế và đưa ra khái niệm về “thời đại hiện nay”, nhấn mạnh thời đại quá độ từ chủ nghĩa tư bản lên chủ nghĩa xã hội trên phạm vi toàn thế giới
-- Hội nghị thông qua bản Tuyên ngôn mới, bổ sung và phát triển nội dung Tuyên ngôn năm 1957, được coi là cương lĩnh cách mạng chung cho các Đảng Mác – Lênin trên thế giới</t>
+    <t xml:space="preserve">- Hội nghị đại biểu của 81 Đảng Cộng sản và Đảng Công nhân quốc tế họp ở Moskva tháng 11/1960, phân tích tình hình quốc tế và đưa ra khái niệm về “thời đại hiện nay”, nhấn mạnh thời đại quá độ từ chủ nghĩa tư bản lên chủ nghĩa xã hội trên phạm vi toàn thế giới.
+- Hội nghị thông qua bản Tuyên ngôn mới, bổ sung và phát triển nội dung Tuyên ngôn năm 1957, được coi là cương lĩnh cách mạng chung cho các Đảng Mác – Lênin trên thế giới.</t>
   </si>
   <si>
-    <t>https://tulieuvankien.dangcongsan.vn/ho-so-su-kien-nhan-chung/su-kien-va-nhan-chung/hoi-nghi-dai-bieu-cac-dang-cong-san-va-dang-cong-nhan-thang-11-1957-tai-matxcova-nga-3370</t>
+    <t>https://tulieuvankien.dangcongsan.vn/ho-so-su-kien-nhan-chung/su-kien-va-nhan-chung/hoi-nghi-dai-bieu-cac-dang-cong-san-va-dang-cong-nhan-thang-11-1960-tai-matxcova-nga-3374</t>
   </si>
   <si>
     <t>https://tse2.mm.bing.net/th/id/OIP.Zoxed5-nMtfNJ8Lp_NlMNgHaD4?r=0&amp;rs=1&amp;pid=ImgDetMain&amp;o=7&amp;rm=3</t>
@@ -546,11 +538,11 @@
     <t>Mô hình chế độ XHCN ở Liên Xô và Đông Âu sụp đổ, hệ thống XHCN tan rã.</t>
   </si>
   <si>
-    <t xml:space="preserve">- Cuối thập niên 1980, cải tổ (perestroika) và công khai (glasnost) ở Liên Xô cùng với khủng hoảng kinh tế – xã hội dẫn tới mất ổn định chính trị, làm suy yếu hệ thống XHCN
-- Năm 1989, các chế độ XHCN Đông Âu lần lượt sụp đổ; đến cuối năm 1991, Liên Xô tan rã, hệ thống xã hội chủ nghĩa thế giới bị thu hẹp mạnh, chỉ còn một số nước như Trung Quốc, Việt Nam, Cuba, Lào, Bắc Triều Tiên tiếp tục con đường XHCN</t>
+    <t xml:space="preserve">- Cuối thập niên 1980, cải tổ (perestroika) và công khai (glasnost) ở Liên Xô cùng với khủng hoảng kinh tế – xã hội dẫn tới mất ổn định chính trị, làm suy yếu hệ thống XHCN.
+- Năm 1989, các chế độ XHCN Đông Âu lần lượt sụp đổ; đến cuối năm 1991, Liên Xô tan rã, hệ thống xã hội chủ nghĩa thế giới bị thu hẹp mạnh, chỉ còn một số nước như Trung Quốc, Việt Nam, Cuba, Lào, Bắc Triều Tiên tiếp tục con đường XHCN.</t>
   </si>
   <si>
-    <t>https://tapchilichsudang.vn/mot-so-yeu-to-tac-dong-den-su-hinh-thanh-duong-loi-xay-dung-chu-nghia-xa-hoi-o-mien-bac-1954-1975.html</t>
+    <t>https://nhandan.vn/bai-hoc-tu-su-sup-do-cua-chu-nghia-xa-hoi-o-lien-xo-va-dong-au-post308642.html</t>
   </si>
   <si>
     <t>https://th.bing.com/th/id/OIP.68mwPoMFrCywyIE5tr6j7AHaFl?w=312&amp;h=200&amp;c=10&amp;o=6&amp;pid=genserp&amp;rm=2</t>
@@ -559,30 +551,27 @@
     <t>08/11/2002 - 14/11/2002</t>
   </si>
   <si>
-    <t>08/11/2002Đại lễ đường Nhân dân, Bắc Kinh, Trung Quốc</t>
+    <t>Đại lễ đường Nhân dân, Bắc Kinh, Trung Quốc</t>
   </si>
   <si>
     <t>Đại hội lần thứ XVI Đảng Cộng sản Trung Quốc khái quát về quá trình lãnh đạo của Đảng.</t>
   </si>
   <si>
-    <t xml:space="preserve">- Đại hội XVI đã tổng kết quá trình lãnh đạo của Đảng Cộng sản Trung Quốc trong giai đoạn cải cách – mở cửa, xác lập tư tưởng “Ba đại diện” là cơ sở lý luận quan trọng để CPC tiếp tục cầm quyền trong điều kiện kinh tế thị trường xã hội chủ nghĩa
+    <t xml:space="preserve">- Đại hội XVI đã tổng kết quá trình lãnh đạo của Đảng Cộng sản Trung Quốc trong giai đoạn cải cách – mở cửa, xác lập tư tưởng “Ba đại diện” là cơ sở lý luận quan trọng để CPC tiếp tục cầm quyền trong điều kiện kinh tế thị trường xã hội chủ nghĩa.
 - Đại hội đề ra mục tiêu tiếp tục hiện đại hóa, thúc đẩy công nghiệp hóa, đô thị hóa và hội nhập kinh tế quốc tế, vừa củng cố vai trò lãnh đạo của Đảng, vừa mở rộng thành phần kinh tế ngoài quốc doanh.</t>
   </si>
   <si>
     <t>https://vi.wikipedia.org/wiki/%C4%90%E1%BA%A1i_h%E1%BB%99i_%C4%90%E1%BA%A3ng_C%E1%BB%99ng_s%E1%BA%A3n_Trung_Qu%E1%BB%91c_l%E1%BA%A7n_th%E1%BB%A9_XVI</t>
   </si>
   <si>
-    <t xml:space="preserve"> 18/10/2017 - 24/10/2017.</t>
-  </si>
-  <si>
-    <t>Đại lễ đường Nhân dân, Bắc Kinh, Trung Quố</t>
+    <t>18/10/2017 - 24/10/2017</t>
   </si>
   <si>
     <t>Đại hội XIX của Đảng Cộng sản Trung Quốc xác lập tư tưởng về chủ nghĩa xã hội đặc sắc Trung Quốc thời đại mới.</t>
   </si>
   <si>
     <t xml:space="preserve">- Đại hội XIX xác lập “Tư tưởng về chủ nghĩa xã hội đặc sắc Trung Quốc trong thời đại mới” của Tập Cận Bình, đưa tư tưởng này vào Cương lĩnh Đảng, khẳng định bước phát triển mới của mô hình XHCN mang đặc sắc Trung Quốc.
-- Đại hội đề ra mục tiêu đến giữa thế kỷ XXI xây dựng Trung Quốc trở thành nước xã hội chủ nghĩa hiện đại toàn diện, đồng thời nhấn mạnh vai trò lãnh đạo toàn diện của Đảng trong mọi lĩnh vực</t>
+- Đại hội đề ra mục tiêu đến giữa thế kỷ XXI xây dựng Trung Quốc trở thành nước xã hội chủ nghĩa hiện đại toàn diện, đồng thời nhấn mạnh vai trò lãnh đạo toàn diện của Đảng trong mọi lĩnh vực.</t>
   </si>
   <si>
     <t>https://baotintuc.vn/phan-tichnhan-dinh/dai-hoi-xix-cua-dang-cong-san-trung-quoc-diem-khoi-dau-lich-su-moi-cua-trung-quoc-20171021102418925.htm</t>
@@ -600,7 +589,7 @@
     <t>Hương Cảng (Hong Kong, Trung Quốc)</t>
   </si>
   <si>
-    <t>22.3530245,113.8090476</t>
+    <t>22.3193, 114.1694</t>
   </si>
   <si>
     <t>Cương lĩnh đầu tiên của Đảng Cộng sản Việt Nam xác định con đường đi lên chủ nghĩa xã hội.</t>
@@ -609,7 +598,7 @@
     <t>Hội nghị thành lập Đảng do Nguyễn Ái Quốc chủ trì thông qua Chánh cương vắn tắt, Sách lược vắn tắt…; xác định con đường cách mạng Việt Nam là làm tư sản dân quyền cách mạng và thổ địa cách mạng để đi tới xã hội cộng sản.</t>
   </si>
   <si>
-    <t>https://nhandan.vn/cuong-linh-xay-dung-dat-nuoc-trong-thoi-ky-qua-do-len-chu-nghia-xa-hoi-post935095.html?</t>
+    <t>https://tulieuvankien.dangcongsan.vn/ho-so-su-kien-nhan-chung/su-kien-va-nhan-chung/ngay-thanh-lap-dang-cong-san-viet-nam-3-2-1930-3342</t>
   </si>
   <si>
     <t>https://thanhuyhanoi.vn/tin-tuc/xay-dung-dang/cuong-linh-chinh-tri-dau-tien-cua-dang-va-khat-vong-doc-lap-tu-do-hanh-phuc-10024770.html</t>
@@ -630,7 +619,7 @@
     <t>Cách mạng Tháng Tám giành chính quyền trên cả nước, chấm dứt chế độ thực dân - phong kiến; ngày 02/9/1945, Chủ tịch Hồ Chí Minh đọc Tuyên ngôn Độc lập, khai sinh nước Việt Nam Dân chủ Cộng hòa.</t>
   </si>
   <si>
-    <t>https://nhandan.vn/cuong-linh-xay-dung-dat-nuoc-trong-thoi-ky-qua-do-len-chu-nghia-xa-hoi-post935095.html</t>
+    <t>https://tulieuvankien.dangcongsan.vn/ho-so-su-kien-nhan-chung/su-kien-va-nhan-chung/cach-mang-thang-8-va-quoc-khanh-291945-cua-nuoc-viet-nam-dan-chu-cong-hoa-3310</t>
   </si>
   <si>
     <t>https://thegioidisan.vn/vi/cach-mang-thang-tam-suy-nghi-va-cam-nhan.html</t>
@@ -651,7 +640,7 @@
     <t>Hà Nội (Kỳ họp thứ nhất Quốc hội khóa VI)</t>
   </si>
   <si>
-    <t>20.9751749,105.3223869</t>
+    <t>21.0367, 105.8347</t>
   </si>
   <si>
     <t>Tên nước được đổi thành Cộng hòa xã hội chủ nghĩa Việt Nam.</t>
@@ -693,7 +682,7 @@
     <t>Thông qua Cương lĩnh xây dựng đất nước trong thời kỳ quá độ lên chủ nghĩa xã hội.</t>
   </si>
   <si>
-    <t>Đại hội VII thông qua Cương lĩnh năm 1991, xác định mô hình xã hội xã hội chủ nghĩa và phương hướng xây dựng đất nước trong thời kỳ quá độ</t>
+    <t>Đại hội VII thông qua Cương lĩnh năm 1991, xác định mô hình xã hội xã hội chủ nghĩa và phương hướng xây dựng đất nước trong thời kỳ quá độ.</t>
   </si>
   <si>
     <t>https://dantri.com.vn/thoi-su/dai-hoi-vii-cua-dang-dua-dat-nuoc-di-theo-con-duong-doi-moi-20260115152225377.htm</t>
@@ -702,13 +691,16 @@
     <t>12–19/01/2011</t>
   </si>
   <si>
+    <t>21.0043, 105.7871</t>
+  </si>
+  <si>
     <t>Thông qua Cương lĩnh (bổ sung, phát triển năm 2011) tại Đại hội XI</t>
   </si>
   <si>
     <t>Đại hội XI thông qua Cương lĩnh xây dựng đất nước trong thời kỳ quá độ lên CNXH (bổ sung, phát triển năm 2011); bổ sung nhiều nội dung về đặc trưng xã hội xã hội chủ nghĩa và phương hướng phát triển đất nước.</t>
   </si>
   <si>
-    <t>https://dcs.nhandan.vn/tu-lieu-tham-khao-cuoc-thi-trac-nghiem-tim-hieu-90-nam-lich-su-ve-vang-cua-dang-cong-san-viet-nam/tu-lieu-cuoc-thi/cuong-linh-xay-dung-dat-nuoc-trong-thoi-ky-qua-do-len-chu-nghia-xa-hoi-nam-1991-543533.html</t>
+    <t>https://tulieuvankien.dangcongsan.vn/ban-chap-hanh-trung-uong-dang/dai-hoi-dang/lan-thu-xi/cuong-linh-xay-dung-dat-nuoc-trong-thoi-ky-qua-do-len-chu-nghia-xa-hoi-bo-sung-phat-trien-nam-2011-1528</t>
   </si>
   <si>
     <t>https://cdcsnd1.bocongan.gov.vn/home/nghien-cuu-trao-doi/cuong-linh-2011-cua-dang-cong-san-viet-nam-voi-xu-the-thoi-dai-298</t>
@@ -2585,22 +2577,22 @@
         <v>170</v>
       </c>
       <c r="C29" s="19" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="D29" s="19" t="s">
         <v>154</v>
       </c>
       <c r="E29" s="19" t="s">
+        <v>171</v>
+      </c>
+      <c r="F29" s="19" t="s">
         <v>172</v>
       </c>
-      <c r="F29" s="19" t="s">
+      <c r="G29" s="20" t="s">
         <v>173</v>
       </c>
-      <c r="G29" s="20" t="s">
+      <c r="H29" s="36" t="s">
         <v>174</v>
-      </c>
-      <c r="H29" s="36" t="s">
-        <v>175</v>
       </c>
       <c r="I29" s="22"/>
       <c r="J29" s="9"/>
@@ -2624,7 +2616,7 @@
     </row>
     <row r="30" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B30" s="6"/>
       <c r="C30" s="6"/>
@@ -2656,25 +2648,25 @@
     <row r="31" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A31" s="10"/>
       <c r="B31" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="C31" s="37" t="s">
         <v>177</v>
       </c>
-      <c r="C31" s="37" t="s">
+      <c r="D31" s="38" t="s">
         <v>178</v>
       </c>
-      <c r="D31" s="38" t="s">
+      <c r="E31" s="39" t="s">
         <v>179</v>
       </c>
-      <c r="E31" s="39" t="s">
+      <c r="F31" s="11" t="s">
         <v>180</v>
       </c>
-      <c r="F31" s="11" t="s">
+      <c r="G31" s="12" t="s">
         <v>181</v>
       </c>
-      <c r="G31" s="12" t="s">
+      <c r="H31" s="13" t="s">
         <v>182</v>
-      </c>
-      <c r="H31" s="13" t="s">
-        <v>183</v>
       </c>
       <c r="I31" s="14"/>
       <c r="J31" s="9"/>
@@ -2699,25 +2691,25 @@
     <row r="32" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A32" s="10"/>
       <c r="B32" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="C32" s="37" t="s">
         <v>184</v>
       </c>
-      <c r="C32" s="37" t="s">
+      <c r="D32" s="38" t="s">
         <v>185</v>
       </c>
-      <c r="D32" s="38" t="s">
+      <c r="E32" s="39" t="s">
         <v>186</v>
       </c>
-      <c r="E32" s="39" t="s">
+      <c r="F32" s="11" t="s">
         <v>187</v>
       </c>
-      <c r="F32" s="11" t="s">
+      <c r="G32" s="12" t="s">
         <v>188</v>
       </c>
-      <c r="G32" s="12" t="s">
+      <c r="H32" s="13" t="s">
         <v>189</v>
-      </c>
-      <c r="H32" s="13" t="s">
-        <v>190</v>
       </c>
       <c r="I32" s="14"/>
       <c r="J32" s="9"/>
@@ -2745,22 +2737,22 @@
         <v>16808</v>
       </c>
       <c r="C33" s="37" t="s">
+        <v>190</v>
+      </c>
+      <c r="D33" s="39" t="s">
+        <v>185</v>
+      </c>
+      <c r="E33" s="39" t="s">
         <v>191</v>
       </c>
-      <c r="D33" s="39" t="s">
-        <v>186</v>
-      </c>
-      <c r="E33" s="39" t="s">
+      <c r="F33" s="11" t="s">
         <v>192</v>
       </c>
-      <c r="F33" s="11" t="s">
+      <c r="G33" s="40" t="s">
         <v>193</v>
       </c>
-      <c r="G33" s="40" t="s">
-        <v>194</v>
-      </c>
       <c r="H33" s="13" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="I33" s="14"/>
       <c r="J33" s="9"/>
@@ -2788,22 +2780,22 @@
         <v>27943</v>
       </c>
       <c r="C34" s="37" t="s">
+        <v>194</v>
+      </c>
+      <c r="D34" s="38" t="s">
         <v>195</v>
       </c>
-      <c r="D34" s="38" t="s">
+      <c r="E34" s="39" t="s">
         <v>196</v>
       </c>
-      <c r="E34" s="39" t="s">
+      <c r="F34" s="11" t="s">
         <v>197</v>
       </c>
-      <c r="F34" s="11" t="s">
+      <c r="G34" s="40" t="s">
         <v>198</v>
       </c>
-      <c r="G34" s="40" t="s">
+      <c r="H34" s="13" t="s">
         <v>199</v>
-      </c>
-      <c r="H34" s="13" t="s">
-        <v>200</v>
       </c>
       <c r="I34" s="14"/>
       <c r="J34" s="9"/>
@@ -2828,25 +2820,25 @@
     <row r="35" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A35" s="10"/>
       <c r="B35" s="41" t="s">
+        <v>200</v>
+      </c>
+      <c r="C35" s="37" t="s">
         <v>201</v>
       </c>
-      <c r="C35" s="37" t="s">
+      <c r="D35" s="38" t="s">
+        <v>195</v>
+      </c>
+      <c r="E35" s="38" t="s">
         <v>202</v>
       </c>
-      <c r="D35" s="38" t="s">
-        <v>196</v>
-      </c>
-      <c r="E35" s="38" t="s">
+      <c r="F35" s="11" t="s">
         <v>203</v>
       </c>
-      <c r="F35" s="11" t="s">
+      <c r="G35" s="40" t="s">
         <v>204</v>
       </c>
-      <c r="G35" s="40" t="s">
+      <c r="H35" s="13" t="s">
         <v>205</v>
-      </c>
-      <c r="H35" s="13" t="s">
-        <v>206</v>
       </c>
       <c r="I35" s="14"/>
       <c r="J35" s="9"/>
@@ -2871,25 +2863,25 @@
     <row r="36" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A36" s="24"/>
       <c r="B36" s="42" t="s">
+        <v>206</v>
+      </c>
+      <c r="C36" s="43" t="s">
         <v>207</v>
       </c>
-      <c r="C36" s="43" t="s">
+      <c r="D36" s="44" t="s">
+        <v>195</v>
+      </c>
+      <c r="E36" s="39" t="s">
         <v>208</v>
       </c>
-      <c r="D36" s="44" t="s">
-        <v>196</v>
-      </c>
-      <c r="E36" s="39" t="s">
+      <c r="F36" s="26" t="s">
         <v>209</v>
       </c>
-      <c r="F36" s="26" t="s">
+      <c r="G36" s="45" t="s">
         <v>210</v>
       </c>
-      <c r="G36" s="45" t="s">
-        <v>211</v>
-      </c>
       <c r="H36" s="28" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="I36" s="46"/>
       <c r="J36" s="9"/>
@@ -2914,13 +2906,13 @@
     <row r="37" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A37" s="24"/>
       <c r="B37" s="42" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C37" s="26" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D37" s="26" t="s">
-        <v>196</v>
+        <v>212</v>
       </c>
       <c r="E37" s="26" t="s">
         <v>213</v>
@@ -2960,10 +2952,10 @@
         <v>217</v>
       </c>
       <c r="C38" s="19" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D38" s="19" t="s">
-        <v>196</v>
+        <v>212</v>
       </c>
       <c r="E38" s="19" t="s">
         <v>218</v>
@@ -31454,85 +31446,68 @@
     <mergeCell ref="A30:H30"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="G3" r:id="rId1"/>
-    <hyperlink ref="H3" r:id="rId2"/>
-    <hyperlink ref="G4" r:id="rId3"/>
-    <hyperlink ref="H4" r:id="rId4"/>
-    <hyperlink ref="G5" r:id="rId5"/>
-    <hyperlink ref="H5" r:id="rId6"/>
-    <hyperlink ref="G6" r:id="rId7"/>
-    <hyperlink ref="H6" r:id="rId8"/>
-    <hyperlink ref="G7" r:id="rId9"/>
-    <hyperlink ref="H7" r:id="rId10"/>
-    <hyperlink ref="G8" r:id="rId11"/>
-    <hyperlink ref="H8" r:id="rId12"/>
-    <hyperlink ref="G9" r:id="rId13"/>
-    <hyperlink ref="H9" r:id="rId14"/>
-    <hyperlink ref="G10" r:id="rId15"/>
-    <hyperlink ref="H10" r:id="rId16"/>
-    <hyperlink ref="G11" r:id="rId17"/>
-    <hyperlink ref="H11" r:id="rId18"/>
-    <hyperlink ref="G12" r:id="rId19"/>
-    <hyperlink ref="H12" r:id="rId20"/>
-    <hyperlink ref="G13" r:id="rId21"/>
-    <hyperlink ref="H13" r:id="rId22"/>
-    <hyperlink ref="G15" r:id="rId23"/>
-    <hyperlink ref="H15" r:id="rId24"/>
-    <hyperlink ref="I15" r:id="rId25"/>
-    <hyperlink ref="G16" r:id="rId26"/>
-    <hyperlink ref="H16" r:id="rId27"/>
-    <hyperlink ref="I16" r:id="rId28"/>
-    <hyperlink ref="G17" r:id="rId29"/>
-    <hyperlink ref="H17" r:id="rId30"/>
-    <hyperlink ref="I17" r:id="rId31"/>
-    <hyperlink ref="G18" r:id="rId32"/>
-    <hyperlink ref="H18" r:id="rId33"/>
-    <hyperlink ref="I18" r:id="rId34"/>
-    <hyperlink ref="G19" r:id="rId35"/>
-    <hyperlink ref="H19" r:id="rId36"/>
-    <hyperlink ref="I19" r:id="rId37"/>
-    <hyperlink ref="C20" r:id="rId38"/>
-    <hyperlink ref="G20" r:id="rId39"/>
-    <hyperlink ref="H20" r:id="rId40"/>
-    <hyperlink ref="I20" r:id="rId41"/>
-    <hyperlink ref="G22" r:id="rId42"/>
-    <hyperlink ref="H22" r:id="rId43"/>
-    <hyperlink ref="I22" r:id="rId44"/>
-    <hyperlink ref="G23" r:id="rId45"/>
-    <hyperlink ref="H23" r:id="rId46"/>
-    <hyperlink ref="I23" r:id="rId47"/>
-    <hyperlink ref="G24" r:id="rId48"/>
-    <hyperlink ref="H24" r:id="rId49"/>
-    <hyperlink ref="G25" r:id="rId50"/>
-    <hyperlink ref="H25" r:id="rId51"/>
-    <hyperlink ref="G26" r:id="rId52"/>
-    <hyperlink ref="H26" r:id="rId53"/>
-    <hyperlink ref="G27" r:id="rId54"/>
-    <hyperlink ref="H27" r:id="rId55"/>
-    <hyperlink ref="G28" r:id="rId56"/>
-    <hyperlink ref="H28" r:id="rId57"/>
-    <hyperlink ref="G29" r:id="rId58"/>
-    <hyperlink ref="H29" r:id="rId59"/>
-    <hyperlink ref="G31" r:id="rId60"/>
-    <hyperlink ref="H31" r:id="rId61"/>
-    <hyperlink ref="G32" r:id="rId62"/>
-    <hyperlink ref="H32" r:id="rId63"/>
-    <hyperlink ref="G33" r:id="rId64"/>
-    <hyperlink ref="H33" r:id="rId65"/>
-    <hyperlink ref="G34" r:id="rId66"/>
-    <hyperlink ref="H34" r:id="rId67"/>
-    <hyperlink ref="G35" r:id="rId68"/>
-    <hyperlink ref="H35" r:id="rId69"/>
-    <hyperlink ref="G36" r:id="rId70"/>
-    <hyperlink ref="H36" r:id="rId71"/>
-    <hyperlink ref="G37" r:id="rId72"/>
-    <hyperlink ref="H37" r:id="rId73"/>
-    <hyperlink ref="G38" r:id="rId74"/>
-    <hyperlink ref="H38" r:id="rId75"/>
+    <hyperlink ref="H3" r:id="rId1"/>
+    <hyperlink ref="H4" r:id="rId2"/>
+    <hyperlink ref="H5" r:id="rId3"/>
+    <hyperlink ref="H6" r:id="rId4"/>
+    <hyperlink ref="H7" r:id="rId5"/>
+    <hyperlink ref="H8" r:id="rId6"/>
+    <hyperlink ref="H9" r:id="rId7"/>
+    <hyperlink ref="H10" r:id="rId8"/>
+    <hyperlink ref="G11" r:id="rId9"/>
+    <hyperlink ref="H11" r:id="rId10"/>
+    <hyperlink ref="G12" r:id="rId11"/>
+    <hyperlink ref="H12" r:id="rId12"/>
+    <hyperlink ref="H13" r:id="rId13"/>
+    <hyperlink ref="G15" r:id="rId14"/>
+    <hyperlink ref="H15" r:id="rId15"/>
+    <hyperlink ref="I15" r:id="rId16"/>
+    <hyperlink ref="G16" r:id="rId17"/>
+    <hyperlink ref="H16" r:id="rId18"/>
+    <hyperlink ref="I16" r:id="rId19"/>
+    <hyperlink ref="G17" r:id="rId20"/>
+    <hyperlink ref="H17" r:id="rId21"/>
+    <hyperlink ref="I17" r:id="rId22"/>
+    <hyperlink ref="G18" r:id="rId23"/>
+    <hyperlink ref="H18" r:id="rId24"/>
+    <hyperlink ref="I18" r:id="rId25"/>
+    <hyperlink ref="G19" r:id="rId26"/>
+    <hyperlink ref="H19" r:id="rId27"/>
+    <hyperlink ref="I19" r:id="rId28"/>
+    <hyperlink ref="G20" r:id="rId29"/>
+    <hyperlink ref="H20" r:id="rId30"/>
+    <hyperlink ref="I20" r:id="rId31"/>
+    <hyperlink ref="H22" r:id="rId32"/>
+    <hyperlink ref="I22" r:id="rId33"/>
+    <hyperlink ref="G23" r:id="rId34"/>
+    <hyperlink ref="H23" r:id="rId35"/>
+    <hyperlink ref="I23" r:id="rId36"/>
+    <hyperlink ref="H24" r:id="rId37"/>
+    <hyperlink ref="H25" r:id="rId38"/>
+    <hyperlink ref="G26" r:id="rId39"/>
+    <hyperlink ref="H26" r:id="rId40"/>
+    <hyperlink ref="H27" r:id="rId41"/>
+    <hyperlink ref="G28" r:id="rId42"/>
+    <hyperlink ref="H28" r:id="rId43"/>
+    <hyperlink ref="G29" r:id="rId44"/>
+    <hyperlink ref="H29" r:id="rId45"/>
+    <hyperlink ref="H31" r:id="rId46"/>
+    <hyperlink ref="H32" r:id="rId47"/>
+    <hyperlink ref="G33" r:id="rId48"/>
+    <hyperlink ref="H33" r:id="rId49"/>
+    <hyperlink ref="G34" r:id="rId50"/>
+    <hyperlink ref="H34" r:id="rId51"/>
+    <hyperlink ref="G35" r:id="rId52"/>
+    <hyperlink ref="H35" r:id="rId53"/>
+    <hyperlink ref="G36" r:id="rId54"/>
+    <hyperlink ref="H36" r:id="rId55"/>
+    <hyperlink ref="H37" r:id="rId56"/>
+    <hyperlink ref="G38" r:id="rId57"/>
+    <hyperlink ref="H38" r:id="rId58"/>
   </hyperlinks>
   <printOptions gridLines="1" horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" pageOrder="overThenDown" cellComments="atEnd" scale="100" fitToWidth="1" fitToHeight="0" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
-  <legacyDrawing r:id="rId77"/>
+  <legacyDrawing r:id="rId60"/>
 </worksheet>
 </file>
</xml_diff>